<commit_message>
brief description of what changed
</commit_message>
<xml_diff>
--- a/curriculum-2026.xlsx
+++ b/curriculum-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pragatidahal/dspg-2026-curriculum-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B9FB07-3819-9142-BC2F-712B2EA14462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98B45EF-64A3-584F-A27E-68EF9EFC7606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8120" yWindow="600" windowWidth="20680" windowHeight="16240" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
+    <workbookView xWindow="8120" yWindow="600" windowWidth="20680" windowHeight="16240" activeTab="1" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -1270,10 +1270,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79ABCE58-A8F1-4047-AD55-074F18A4BD46}">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.1640625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="60.83203125" style="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="72.1640625" style="9" customWidth="1"/>
     <col min="3" max="3" width="18.6640625" style="9" customWidth="1"/>
     <col min="4" max="4" width="16.1640625" style="9" customWidth="1"/>
@@ -1587,12 +1587,14 @@
       <c r="A41" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B41" s="9" t="s">
+    </row>
+    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="9" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="9" t="s">
+    <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="9" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2193,12 +2195,12 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B54" t="s">
+      <c r="A54" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B55" t="s">
+      <c r="A55" t="s">
         <v>123</v>
       </c>
     </row>
@@ -3069,18 +3071,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3102,18 +3104,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
regenerate with all fixes
</commit_message>
<xml_diff>
--- a/curriculum-2026.xlsx
+++ b/curriculum-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chunbeiwang\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pragatidahal/dspg-2026-curriculum-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1173" documentId="13_ncr:1_{65F6ACF4-0E11-4456-A716-D1BBD8106E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31698AAF-FD04-4466-9B80-BC349D3B273E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{963588D3-C371-694A-9249-80352D5ACEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15980" yWindow="580" windowWidth="20680" windowHeight="20730" firstSheet="5" activeTab="5" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -60,9 +60,6 @@
     <t>Week 1</t>
   </si>
   <si>
-    <t>Onboarding and Basic Research skills</t>
-  </si>
-  <si>
     <t>Onboarding and Project Assignment</t>
   </si>
   <si>
@@ -776,12 +773,15 @@
   <si>
     <t>Timing : 9 - 11</t>
   </si>
+  <si>
+    <t xml:space="preserve">Onboarding </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1301,17 +1301,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85F7D784-1E42-A348-A9E2-F410F7914403}">
   <dimension ref="A2:D22"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.625" style="1"/>
-    <col min="2" max="2" width="61.75" style="1" customWidth="1"/>
-    <col min="3" max="3" width="48.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.25" style="1" customWidth="1"/>
-    <col min="5" max="5" width="47.875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.625" style="1"/>
+    <col min="1" max="1" width="10.6640625" style="1"/>
+    <col min="2" max="2" width="61.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="48.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47.83203125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1322,108 +1322,108 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="1" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="1" t="s">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="1" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="1" t="s">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="1" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="1" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="1" t="s">
+    </row>
+    <row r="22" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="30.75">
-      <c r="A22" s="1" t="s">
+      <c r="B22" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1437,7 +1437,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D97929D-AD65-4CE9-BF8E-66086023685B}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1446,7 +1446,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74299BF2-7816-4D37-8F2E-A4AEC8FE33CF}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1455,51 +1455,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79ABCE58-A8F1-4047-AD55-074F18A4BD46}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.25" style="9" customWidth="1"/>
-    <col min="2" max="2" width="72.125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="18.75" style="9" customWidth="1"/>
-    <col min="4" max="4" width="16.125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="40.75" style="9" customWidth="1"/>
-    <col min="6" max="6" width="13.75" style="9" customWidth="1"/>
-    <col min="7" max="16384" width="10.625" style="9"/>
+    <col min="1" max="1" width="21.1640625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="72.1640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="40.6640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" style="9" customWidth="1"/>
+    <col min="7" max="16384" width="10.6640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="8"/>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="9" t="s">
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="C4" s="12">
         <v>0.52083333333333337</v>
@@ -1508,139 +1508,139 @@
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6"/>
-    <row r="6" spans="1:6">
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>40</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="8" spans="1:6" ht="21.75" customHeight="1">
+    <row r="8" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>41</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>42</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
     </row>
-    <row r="9" spans="1:6" ht="21.75" customHeight="1">
+    <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="15"/>
       <c r="B9" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" ht="148.5" customHeight="1">
+    <row r="10" spans="1:6" ht="148.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="15"/>
       <c r="B10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="E10" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="18" t="s">
+    </row>
+    <row r="11" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="18" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="33" customHeight="1">
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="E11" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="9" t="s">
+    </row>
+    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="9" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1">
-      <c r="B12" s="9" t="s">
+      <c r="C12" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="9" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="16" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" customHeight="1"/>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1">
-      <c r="B14" s="16" t="s">
-        <v>53</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="E15" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E15" s="9" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="18" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="63" customHeight="1">
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="20.25" customHeight="1">
+    </row>
+    <row r="17" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18"/>
       <c r="C17" s="19"/>
     </row>
-    <row r="18" spans="1:7" ht="21" customHeight="1">
+    <row r="18" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>60</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>61</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="20"/>
       <c r="F20" s="13"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="21"/>
       <c r="B21" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -1648,183 +1648,183 @@
       <c r="F21" s="16"/>
       <c r="G21" s="21"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="21"/>
       <c r="B22" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" s="21"/>
       <c r="E22" s="21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="21"/>
       <c r="B23" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="E23" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E23" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="21"/>
       <c r="B24" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="E24" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="E24" s="27" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+    </row>
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="21"/>
       <c r="E25" s="22"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="21"/>
       <c r="B26" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="21"/>
       <c r="B27" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="21"/>
       <c r="B28" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="21"/>
+    </row>
+    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="21"/>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="10" t="s">
+      <c r="B30" s="13" t="s">
         <v>74</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>75</v>
       </c>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B31" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B32" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="E32" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E32" s="9" t="s">
+    </row>
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B33" s="9" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="B33" s="9" t="s">
-        <v>79</v>
-      </c>
       <c r="E33" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6"/>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B36" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="E36" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E36" s="9" t="s">
+    </row>
+    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B37" s="9" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="B37" s="9" t="s">
+      <c r="C37" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="E37" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B38" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E37" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="B38" s="9" t="s">
+      <c r="C38" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="E38" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B39" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="E38" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="B39" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C39" s="9" t="s">
+    </row>
+    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="9" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="40" spans="1:6"/>
-    <row r="41" spans="1:6">
-      <c r="A41" s="9" t="s">
+      <c r="B41" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B41" s="9" t="s">
+    </row>
+    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B42" s="9" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1">
-      <c r="B42" s="9" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1835,96 +1835,95 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E724203-93BF-4AB3-BBFF-F621604F3060}">
   <dimension ref="A1:M57"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.625" customWidth="1"/>
-    <col min="2" max="2" width="65.375" customWidth="1"/>
-    <col min="3" max="3" width="18.75" customWidth="1"/>
-    <col min="5" max="5" width="41.625" customWidth="1"/>
-    <col min="6" max="6" width="10.625" customWidth="1"/>
-    <col min="9" max="9" width="30.625" customWidth="1"/>
-    <col min="12" max="12" width="20.75" customWidth="1"/>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="65.33203125" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="41.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
+    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="12" max="12" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75"/>
-    <row r="3" spans="1:6" ht="15.75">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17.25" customHeight="1">
+    <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>93</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>94</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75">
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -1932,45 +1931,45 @@
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -1978,59 +1977,59 @@
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75">
+    <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="15"/>
       <c r="B14" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:13" ht="15.75">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -2038,45 +2037,45 @@
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:13" ht="15.75">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
     </row>
-    <row r="19" spans="1:13" ht="15.75">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:13" ht="15.75">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:13" ht="15.75">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="18"/>
       <c r="C21" s="19"/>
@@ -2084,12 +2083,12 @@
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:13" ht="15.75">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>108</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>109</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -2097,47 +2096,47 @@
       <c r="F22" s="13"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" ht="15.75">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
     </row>
-    <row r="24" spans="1:13" ht="15.75">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:13" ht="15.75">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:13" ht="15.75">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -2145,45 +2144,45 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:13" ht="15.75">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:13" ht="15.75">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:13" ht="15.75">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:13" ht="15.75">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -2191,12 +2190,12 @@
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:13" ht="15.75">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>112</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>113</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
@@ -2204,48 +2203,48 @@
       <c r="F31" s="13"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="1:13" ht="15.75">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="21"/>
       <c r="B32" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:13" ht="15.75">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D33" s="21"/>
       <c r="E33" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F33" s="21"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="1:13" ht="15.75">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="21"/>
       <c r="B34" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="E34" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E34" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:13" ht="18.75" customHeight="1">
+    <row r="35" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -2254,45 +2253,45 @@
       <c r="F35" s="9"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="1:13" ht="15.75">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:13" ht="15.75">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:13" ht="15.75">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:13" ht="15.75">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -2300,85 +2299,85 @@
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40" spans="1:13" ht="15.75">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B40" s="13" t="s">
         <v>117</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>118</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
     </row>
-    <row r="41" spans="1:13" ht="15.75">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
       <c r="F41" s="16"/>
     </row>
-    <row r="42" spans="1:13" ht="15.75">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="9"/>
       <c r="B42" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D42" s="21"/>
       <c r="E42" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:13" ht="15.75">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>120</v>
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:13" ht="15.75">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C44" s="9" t="s">
         <v>122</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>123</v>
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F44" s="9"/>
     </row>
-    <row r="45" spans="1:13" ht="15.75">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C45" s="9" t="s">
         <v>125</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>126</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F45" s="9"/>
     </row>
-    <row r="46" spans="1:13" ht="15.75">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -2386,86 +2385,84 @@
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
     </row>
-    <row r="47" spans="1:13" ht="15.75">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="9"/>
       <c r="B47" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
       <c r="F47" s="16"/>
     </row>
-    <row r="48" spans="1:13" ht="15.75">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="9"/>
       <c r="B48" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F48" s="9"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B49" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C49" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E48" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F48" s="9"/>
-    </row>
-    <row r="49" spans="1:5" ht="15.75">
-      <c r="B49" s="9" t="s">
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B50" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="15.75">
-      <c r="B50" s="9" t="s">
-        <v>129</v>
-      </c>
       <c r="C50" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="15.75">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B51" s="9" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="15.75">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B52" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>130</v>
       </c>
-      <c r="C52" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="15.75"/>
-    <row r="54" spans="1:5" ht="15.75"/>
-    <row r="55" spans="1:5" ht="15.75">
-      <c r="A55" t="s">
+      <c r="B55" t="s">
         <v>131</v>
       </c>
-      <c r="B55" t="s">
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.75">
-      <c r="B56" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5">
-      <c r="B57" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2475,107 +2472,107 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4375F624-6CA8-4BD1-8837-D674A15E3640}">
-  <dimension ref="A1:F85"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <dimension ref="A1:F67"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.25" customWidth="1"/>
-    <col min="2" max="2" width="68.375" customWidth="1"/>
-    <col min="3" max="3" width="21.75" customWidth="1"/>
+    <col min="1" max="1" width="33.1640625" customWidth="1"/>
+    <col min="2" max="2" width="68.33203125" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="42.875" customWidth="1"/>
-    <col min="6" max="6" width="14.625" customWidth="1"/>
+    <col min="5" max="5" width="42.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15.75">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75">
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>136</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>137</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75">
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="26" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -2583,97 +2580,97 @@
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="B13" s="25"/>
       <c r="C13" s="25"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75">
+    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>148</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>149</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="C16" s="29" t="s">
         <v>150</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>151</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:6" ht="15.75">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:6" ht="15.75">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -2681,44 +2678,44 @@
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" ht="15.75">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" ht="15.75">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:6" ht="15.75">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="9"/>
       <c r="B22" s="18"/>
       <c r="C22" s="19"/>
@@ -2726,43 +2723,43 @@
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>153</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
     </row>
-    <row r="24" spans="1:6" ht="15.75">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
     </row>
-    <row r="25" spans="1:6" ht="15.75">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:6" ht="15.75">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -2770,44 +2767,44 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:6" ht="15.75">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:6" ht="15.75">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" ht="15.75">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" ht="15.75">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -2815,43 +2812,43 @@
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:6" ht="15.75">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>156</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>157</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
       <c r="E31" s="20"/>
       <c r="F31" s="13"/>
     </row>
-    <row r="32" spans="1:6" ht="15.75">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="21"/>
       <c r="B32" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:6" ht="15.75">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="21"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -2859,44 +2856,44 @@
       <c r="E34" s="22"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F36" s="9"/>
     </row>
-    <row r="37" spans="1:6" ht="15.75">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -2904,56 +2901,56 @@
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B39" s="13" t="s">
         <v>160</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>161</v>
       </c>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
     </row>
-    <row r="40" spans="1:6" ht="15.75">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="9"/>
       <c r="B40" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
     </row>
-    <row r="41" spans="1:6" ht="15.75">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
+        <v>161</v>
+      </c>
+      <c r="C41" t="s">
         <v>162</v>
       </c>
-      <c r="C41" t="s">
-        <v>163</v>
-      </c>
       <c r="E41" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F41" s="9"/>
     </row>
-    <row r="42" spans="1:6" ht="15.75">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="9"/>
       <c r="B42" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:6" ht="15.75">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -2961,57 +2958,52 @@
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" ht="15.75">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C44" s="16"/>
       <c r="D44" s="16"/>
       <c r="E44" s="16"/>
       <c r="F44" s="16"/>
     </row>
-    <row r="45" spans="1:6" ht="15.75">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C45" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F45" s="9"/>
     </row>
-    <row r="46" spans="1:6" ht="15.75">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B46" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="15.75">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="B49" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="B49" s="25" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2" ht="15.75">
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" s="4"/>
     </row>
-    <row r="78" spans="2:2" ht="15.75"/>
-    <row r="79" spans="2:2" ht="15.75"/>
-    <row r="80" spans="2:2" ht="15.75"/>
-    <row r="84" ht="15.75"/>
-    <row r="85" ht="15.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3019,119 +3011,119 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E959A69-B699-4CFA-82E0-7BD72875D037}">
-  <dimension ref="A1:F63"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.375" customWidth="1"/>
+    <col min="1" max="1" width="27.33203125" customWidth="1"/>
     <col min="2" max="2" width="58.5" customWidth="1"/>
-    <col min="3" max="3" width="17.625" customWidth="1"/>
-    <col min="4" max="4" width="9.375" customWidth="1"/>
-    <col min="5" max="5" width="32.625" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="24"/>
     </row>
-    <row r="3" spans="1:6" ht="15.75">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75">
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>169</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>170</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75">
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>171</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>172</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3139,110 +3131,110 @@
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="B13" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
       <c r="B14" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" s="9"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="B16" s="23" t="s">
         <v>176</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>177</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
     </row>
-    <row r="17" spans="1:6" ht="15.75">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
     </row>
-    <row r="18" spans="1:6" ht="15.75">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="15"/>
       <c r="B18" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" ht="15.75">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="15"/>
       <c r="B19" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -3250,160 +3242,160 @@
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" ht="15.75">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
     </row>
-    <row r="22" spans="1:6" ht="15.75">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="9"/>
       <c r="B22" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F23" s="9"/>
     </row>
-    <row r="24" spans="1:6" ht="15.75">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:6" ht="15.75">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:6" ht="15.75">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>181</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>182</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
     </row>
-    <row r="27" spans="1:6" ht="15.75">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:6" ht="15.75">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" ht="15.75">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" ht="15.75">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="16"/>
     </row>
-    <row r="31" spans="1:6" ht="15.75">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="9"/>
       <c r="B31" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F31" s="9"/>
     </row>
-    <row r="32" spans="1:6" ht="15.75">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="9"/>
       <c r="B32" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F32" s="9"/>
     </row>
-    <row r="33" spans="1:6" ht="15.75">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="9"/>
       <c r="B33" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3411,56 +3403,56 @@
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B35" s="13" t="s">
         <v>186</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>187</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
       <c r="E35" s="20"/>
       <c r="F35" s="13"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:6" ht="15.75">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s">
         <v>162</v>
       </c>
-      <c r="C37" t="s">
-        <v>163</v>
-      </c>
       <c r="E37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -3468,44 +3460,44 @@
       <c r="E39" s="22"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40" spans="1:6" ht="15.75">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="21"/>
       <c r="B40" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
     </row>
-    <row r="41" spans="1:6" ht="15.75">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="21"/>
       <c r="B41" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D41" s="9"/>
       <c r="E41" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F41" s="9"/>
     </row>
-    <row r="42" spans="1:6" ht="15.75">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="21"/>
       <c r="B42" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:6" ht="15.75">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="21"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -3513,39 +3505,35 @@
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" ht="15.75">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B44" s="13" t="s">
         <v>189</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>190</v>
       </c>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
     </row>
-    <row r="45" spans="1:6" ht="15.75">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="F45" s="9"/>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>190</v>
+      </c>
+      <c r="B47" t="s">
         <v>191</v>
       </c>
-      <c r="B47" t="s">
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
-      <c r="B48" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="58" ht="15.75"/>
-    <row r="59" ht="15.75"/>
-    <row r="62" ht="15.75"/>
-    <row r="63" ht="15.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3554,217 +3542,217 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29CC185F-F58B-4882-BB6A-99C5A8DAD27D}">
   <dimension ref="A1:J71"/>
-  <sheetFormatPr defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.75" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
     <col min="2" max="2" width="63" customWidth="1"/>
-    <col min="3" max="3" width="23.375" customWidth="1"/>
-    <col min="4" max="4" width="9.625" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="7" max="7" width="55.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="2" spans="1:10"/>
-    <row r="3" spans="1:10">
-      <c r="A3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="10" t="s">
+      <c r="B4" s="23" t="s">
         <v>195</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>196</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>197</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>198</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="45.75">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B12" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
       <c r="B13" s="25"/>
       <c r="C13" s="25"/>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>202</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>203</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="G14" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="G15" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="9"/>
       <c r="B16" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>205</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>206</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="G16" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>208</v>
-      </c>
       <c r="H16" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="B17" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="G17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
       <c r="J17" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3775,347 +3763,347 @@
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="G19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H21" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B22" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G22" s="25"/>
       <c r="H22" s="25"/>
       <c r="J22" s="9"/>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="18"/>
       <c r="C23" s="19"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
     </row>
-    <row r="31" spans="1:10"/>
-    <row r="32" spans="1:10"/>
-    <row r="33" spans="1:5">
+    <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>213</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>214</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
       <c r="E34" s="20"/>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="22"/>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C39" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B40" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C43" s="16"/>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
+        <v>161</v>
+      </c>
+      <c r="C44" t="s">
         <v>162</v>
       </c>
-      <c r="C44" t="s">
-        <v>163</v>
-      </c>
       <c r="E44" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B47" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B48" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C48" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C49" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5"/>
-    <row r="51" spans="1:5"/>
-    <row r="52" spans="1:5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="51" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="52" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>215</v>
+      </c>
+      <c r="B52" t="s">
         <v>216</v>
       </c>
-      <c r="B52" t="s">
+    </row>
+    <row r="53" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="D53" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
-      <c r="D53" t="s">
+    <row r="54" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" t="s">
+      <c r="B54" t="s">
         <v>219</v>
       </c>
-      <c r="B54" t="s">
+    </row>
+    <row r="55" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="55" spans="1:5"/>
-    <row r="56" spans="1:5">
-      <c r="A56" t="s">
+      <c r="B56" t="s">
         <v>221</v>
       </c>
-      <c r="B56" t="s">
+    </row>
+    <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
-      <c r="B57" t="s">
+    <row r="58" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
-      <c r="A58" t="s">
+      <c r="B58" t="s">
         <v>224</v>
       </c>
-      <c r="B58" t="s">
+      <c r="D58" t="s">
         <v>225</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>226</v>
       </c>
-      <c r="E58" t="s">
+    </row>
+    <row r="59" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="D60" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="59" spans="1:5"/>
-    <row r="60" spans="1:5">
-      <c r="D60" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5"/>
-    <row r="62" spans="1:5"/>
-    <row r="63" spans="1:5"/>
-    <row r="64" spans="1:5"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
+    <row r="61" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="62" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="63" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="65" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="66" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="67" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="69" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="70" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="71" ht="16" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4124,43 +4112,43 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C5580AA-63C5-4A17-B275-34DB10D89DEB}">
   <dimension ref="A14:C19"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="52.375" customWidth="1"/>
+    <col min="1" max="1" width="52.33203125" customWidth="1"/>
     <col min="2" max="2" width="35.5" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.75">
-      <c r="A16" t="s">
+      <c r="B16" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="C16" t="s">
         <v>231</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
+      <c r="C18" t="s">
         <v>233</v>
       </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>235</v>
-      </c>
       <c r="C19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -4174,27 +4162,27 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08672E17-9FFE-4DB4-AF66-56E8BA384E79}">
   <dimension ref="A14:D15"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.25" customWidth="1"/>
-    <col min="2" max="2" width="14.875" customWidth="1"/>
-    <col min="4" max="4" width="22.125" customWidth="1"/>
+    <col min="1" max="1" width="24.1640625" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>235</v>
+      </c>
+      <c r="B15" t="s">
+        <v>216</v>
+      </c>
+      <c r="D15" t="s">
         <v>236</v>
-      </c>
-      <c r="B15" t="s">
-        <v>217</v>
-      </c>
-      <c r="D15" t="s">
-        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -4205,7 +4193,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11C2D4C5-F861-4F4B-9751-7CF6281C8800}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4221,6 +4209,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100411B9ADA3C88D84DA852962C88CCCF71" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fb8c17446f1b3f0664823c0cd0cfd6e0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="29555bce-99f7-4351-a06e-6e58a2a8a9c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a69d9eff398ae5b3f2ca614c38d74f66" ns2:_="">
     <xsd:import namespace="29555bce-99f7-4351-a06e-6e58a2a8a9c5"/>
@@ -4358,20 +4352,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C57BA70C-BAC7-4091-B4F1-876342C6970D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C57BA70C-BAC7-4091-B4F1-876342C6970D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="29555bce-99f7-4351-a06e-6e58a2a8a9c5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
bake all fixes into script permanently
</commit_message>
<xml_diff>
--- a/curriculum-2026.xlsx
+++ b/curriculum-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pragatidahal/dspg-2026-curriculum-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chunbeiwang\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{963588D3-C371-694A-9249-80352D5ACEEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1173" documentId="13_ncr:1_{65F6ACF4-0E11-4456-A716-D1BBD8106E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31698AAF-FD04-4466-9B80-BC349D3B273E}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
+    <workbookView xWindow="15980" yWindow="580" windowWidth="20680" windowHeight="20730" firstSheet="5" activeTab="5" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -60,6 +60,9 @@
     <t>Week 1</t>
   </si>
   <si>
+    <t>Onboarding and Basic Research skills</t>
+  </si>
+  <si>
     <t>Onboarding and Project Assignment</t>
   </si>
   <si>
@@ -773,15 +776,12 @@
   <si>
     <t>Timing : 9 - 11</t>
   </si>
-  <si>
-    <t xml:space="preserve">Onboarding </t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1301,17 +1301,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85F7D784-1E42-A348-A9E2-F410F7914403}">
   <dimension ref="A2:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="1"/>
-    <col min="2" max="2" width="61.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="48.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="47.83203125" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.6640625" style="1"/>
+    <col min="1" max="1" width="10.625" style="1"/>
+    <col min="2" max="2" width="61.75" style="1" customWidth="1"/>
+    <col min="3" max="3" width="48.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.25" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47.875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1322,108 +1322,108 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>237</v>
+        <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30.75">
       <c r="A22" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1437,7 +1437,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D97929D-AD65-4CE9-BF8E-66086023685B}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1446,7 +1446,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74299BF2-7816-4D37-8F2E-A4AEC8FE33CF}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1455,51 +1455,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79ABCE58-A8F1-4047-AD55-074F18A4BD46}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="21.1640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="72.1640625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="9" customWidth="1"/>
-    <col min="4" max="4" width="16.1640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="40.6640625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" style="9" customWidth="1"/>
-    <col min="7" max="16384" width="10.6640625" style="9"/>
+    <col min="1" max="1" width="21.25" style="9" customWidth="1"/>
+    <col min="2" max="2" width="72.125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="18.75" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16.125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="40.75" style="9" customWidth="1"/>
+    <col min="6" max="6" width="13.75" style="9" customWidth="1"/>
+    <col min="7" max="16384" width="10.625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1">
       <c r="A2" s="8"/>
     </row>
-    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" s="12">
         <v>0.52083333333333337</v>
@@ -1508,139 +1508,139 @@
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6"/>
+    <row r="6" spans="1:6">
       <c r="A6" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="8" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="21.75" customHeight="1">
       <c r="A8" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
     </row>
-    <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="21.75" customHeight="1">
       <c r="A9" s="15"/>
       <c r="B9" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" ht="148.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="148.5" customHeight="1">
       <c r="A10" s="15"/>
       <c r="B10" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="33" customHeight="1">
       <c r="B11" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="19.5" customHeight="1">
       <c r="B12" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="19.5" customHeight="1"/>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1">
       <c r="B14" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1">
       <c r="B15" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="63" customHeight="1">
       <c r="B16" s="18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="20.25" customHeight="1">
       <c r="B17" s="18"/>
       <c r="C17" s="19"/>
     </row>
-    <row r="18" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="21" customHeight="1">
       <c r="A18" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
     </row>
-    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="20"/>
       <c r="F20" s="13"/>
     </row>
-    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21" s="21"/>
       <c r="B21" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -1648,183 +1648,183 @@
       <c r="F21" s="16"/>
       <c r="G21" s="21"/>
     </row>
-    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7">
       <c r="A22" s="21"/>
       <c r="B22" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D22" s="21"/>
       <c r="E22" s="21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
     </row>
-    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7">
       <c r="A23" s="21"/>
       <c r="B23" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" s="21"/>
       <c r="B24" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" s="21"/>
       <c r="E25" s="22"/>
     </row>
-    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="21"/>
       <c r="B26" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
     </row>
-    <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7">
       <c r="A27" s="21"/>
       <c r="B27" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" s="21"/>
       <c r="B28" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" s="21"/>
     </row>
-    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7">
       <c r="A30" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
     </row>
-    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7">
       <c r="B31" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
     </row>
-    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7">
       <c r="B32" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="B33" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6"/>
+    <row r="35" spans="1:6" ht="15.75" customHeight="1">
       <c r="B35" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="B36" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="B37" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E37" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="1:6">
       <c r="B38" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="B39" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6"/>
+    <row r="41" spans="1:6">
       <c r="A41" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="15.75" customHeight="1">
       <c r="B42" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1835,95 +1835,96 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E724203-93BF-4AB3-BBFF-F621604F3060}">
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" customWidth="1"/>
-    <col min="2" max="2" width="65.33203125" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="41.6640625" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" customWidth="1"/>
-    <col min="9" max="9" width="30.6640625" customWidth="1"/>
-    <col min="12" max="12" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="30.625" customWidth="1"/>
+    <col min="2" max="2" width="65.375" customWidth="1"/>
+    <col min="3" max="3" width="18.75" customWidth="1"/>
+    <col min="5" max="5" width="41.625" customWidth="1"/>
+    <col min="6" max="6" width="10.625" customWidth="1"/>
+    <col min="9" max="9" width="30.625" customWidth="1"/>
+    <col min="12" max="12" width="20.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="24" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75"/>
+    <row r="3" spans="1:6" ht="15.75">
       <c r="A3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="17.25" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="15.75">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="15.75">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="15.75">
       <c r="A7" s="9"/>
       <c r="B7" s="26" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="15.75">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -1931,45 +1932,45 @@
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="15.75">
       <c r="A9" s="9"/>
       <c r="B9" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="15.75">
       <c r="A10" s="9"/>
       <c r="B10" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="15.75">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="15.75">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -1977,59 +1978,59 @@
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="15.75">
       <c r="A13" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="15.75">
       <c r="A14" s="15"/>
       <c r="B14" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="15.75">
       <c r="A15" s="15"/>
       <c r="B15" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="15.75">
       <c r="A16" s="15"/>
       <c r="B16" s="26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="15.75">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -2037,45 +2038,45 @@
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="15.75">
       <c r="A18" s="9"/>
       <c r="B18" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="15.75">
       <c r="A19" s="9"/>
       <c r="B19" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="15.75">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="15.75">
       <c r="A21" s="9"/>
       <c r="B21" s="18"/>
       <c r="C21" s="19"/>
@@ -2083,12 +2084,12 @@
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="15.75">
       <c r="A22" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -2096,47 +2097,47 @@
       <c r="F22" s="13"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="15.75">
       <c r="A23" s="9"/>
       <c r="B23" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="15.75">
       <c r="A24" s="9"/>
       <c r="B24" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="15.75">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="15.75">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -2144,45 +2145,45 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="15.75">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="15.75">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="15.75">
       <c r="A29" s="9"/>
       <c r="B29" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="15.75">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -2190,12 +2191,12 @@
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="15.75">
       <c r="A31" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
@@ -2203,48 +2204,48 @@
       <c r="F31" s="13"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="15.75">
       <c r="A32" s="21"/>
       <c r="B32" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" ht="15.75">
       <c r="A33" s="21"/>
       <c r="B33" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D33" s="21"/>
       <c r="E33" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F33" s="21"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" ht="15.75">
       <c r="A34" s="21"/>
       <c r="B34" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" ht="18.75" customHeight="1">
       <c r="A35" s="21"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -2253,45 +2254,45 @@
       <c r="F35" s="9"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" ht="15.75">
       <c r="A36" s="21"/>
       <c r="B36" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="15.75">
       <c r="A37" s="21"/>
       <c r="B37" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="15.75">
       <c r="A38" s="21"/>
       <c r="B38" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" ht="15.75">
       <c r="A39" s="21"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -2299,85 +2300,85 @@
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" ht="15.75">
       <c r="A40" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="15.75">
       <c r="A41" s="9"/>
       <c r="B41" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
       <c r="F41" s="16"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="15.75">
       <c r="A42" s="9"/>
       <c r="B42" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D42" s="21"/>
       <c r="E42" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" ht="15.75">
       <c r="A43" s="9"/>
       <c r="B43" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" ht="15.75">
       <c r="A44" s="9"/>
       <c r="B44" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F44" s="9"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" ht="15.75">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F45" s="9"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" ht="15.75">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -2385,84 +2386,86 @@
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" ht="15.75">
       <c r="A47" s="9"/>
       <c r="B47" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
       <c r="F47" s="16"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" ht="15.75">
       <c r="A48" s="9"/>
       <c r="B48" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F48" s="9"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" ht="15.75">
       <c r="B49" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.75">
       <c r="B50" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.75">
       <c r="B51" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.75">
       <c r="B52" s="25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C52" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="15.75"/>
+    <row r="54" spans="1:5" ht="15.75"/>
+    <row r="55" spans="1:5" ht="15.75">
       <c r="A55" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B55" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="15.75">
       <c r="B56" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
       <c r="B57" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2472,107 +2475,107 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4375F624-6CA8-4BD1-8837-D674A15E3640}">
-  <dimension ref="A1:F67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F85"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="33.1640625" customWidth="1"/>
-    <col min="2" max="2" width="68.33203125" customWidth="1"/>
-    <col min="3" max="3" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="33.25" customWidth="1"/>
+    <col min="2" max="2" width="68.375" customWidth="1"/>
+    <col min="3" max="3" width="21.75" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="42.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="42.875" customWidth="1"/>
+    <col min="6" max="6" width="14.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75">
       <c r="A3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="15.75">
       <c r="A4" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="15.75">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="15.75">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="15.75">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="15.75">
       <c r="A8" s="9"/>
       <c r="B8" s="26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="15.75">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -2580,97 +2583,97 @@
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="15.75">
       <c r="A10" s="9"/>
       <c r="B10" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="15.75">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="15.75">
       <c r="A12" s="9"/>
       <c r="B12" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="15.75">
       <c r="A13" s="9"/>
       <c r="B13" s="25"/>
       <c r="C13" s="25"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="15.75">
       <c r="A14" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="15.75">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="15.75">
       <c r="A16" s="15"/>
       <c r="B16" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="15.75">
       <c r="A17" s="15"/>
       <c r="B17" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="15.75">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -2678,44 +2681,44 @@
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="15.75">
       <c r="A19" s="9"/>
       <c r="B19" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="15.75">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="15.75">
       <c r="A21" s="9"/>
       <c r="B21" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="15.75">
       <c r="A22" s="9"/>
       <c r="B22" s="18"/>
       <c r="C22" s="19"/>
@@ -2723,43 +2726,43 @@
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="15.75">
       <c r="A23" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="15.75">
       <c r="A24" s="9"/>
       <c r="B24" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="15.75">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="15.75">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -2767,44 +2770,44 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="15.75">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="15.75">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="15.75">
       <c r="A29" s="9"/>
       <c r="B29" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="15.75">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -2812,43 +2815,43 @@
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="15.75">
       <c r="A31" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
       <c r="E31" s="20"/>
       <c r="F31" s="13"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ht="15.75">
       <c r="A32" s="21"/>
       <c r="B32" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="15.75">
       <c r="A33" s="21"/>
       <c r="B33" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="15.75">
       <c r="A34" s="21"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -2856,44 +2859,44 @@
       <c r="E34" s="22"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="15.75">
       <c r="A35" s="21"/>
       <c r="B35" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="15.75">
       <c r="A36" s="21"/>
       <c r="B36" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F36" s="9"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" ht="15.75">
       <c r="A37" s="21"/>
       <c r="B37" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="15.75">
       <c r="A38" s="21"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -2901,56 +2904,56 @@
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="15.75">
       <c r="A39" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ht="15.75">
       <c r="A40" s="9"/>
       <c r="B40" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" ht="15.75">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C41" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E41" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F41" s="9"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="15.75">
       <c r="A42" s="9"/>
       <c r="B42" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" ht="15.75">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -2958,52 +2961,57 @@
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" ht="15.75">
       <c r="A44" s="9"/>
       <c r="B44" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C44" s="16"/>
       <c r="D44" s="16"/>
       <c r="E44" s="16"/>
       <c r="F44" s="16"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="15.75">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F45" s="9"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" ht="15.75">
       <c r="B46" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="15.75">
       <c r="A49" s="25" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B49" s="25" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" ht="15.75">
       <c r="B67" s="4"/>
     </row>
+    <row r="78" spans="2:2" ht="15.75"/>
+    <row r="79" spans="2:2" ht="15.75"/>
+    <row r="80" spans="2:2" ht="15.75"/>
+    <row r="84" ht="15.75"/>
+    <row r="85" ht="15.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3011,119 +3019,119 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E959A69-B699-4CFA-82E0-7BD72875D037}">
-  <dimension ref="A1:F48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F63"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="27.33203125" customWidth="1"/>
+    <col min="1" max="1" width="27.375" customWidth="1"/>
     <col min="2" max="2" width="58.5" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" customWidth="1"/>
-    <col min="5" max="5" width="32.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.625" customWidth="1"/>
+    <col min="4" max="4" width="9.375" customWidth="1"/>
+    <col min="5" max="5" width="32.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="24" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75">
       <c r="A2" s="24"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="15.75">
       <c r="A3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="15.75">
       <c r="A4" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="15.75">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="15.75">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="15.75">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="15.75">
       <c r="A8" s="9"/>
       <c r="B8" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="15.75">
       <c r="A9" s="9"/>
       <c r="B9" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="15.75">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3131,110 +3139,110 @@
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="15.75">
       <c r="A11" s="9"/>
       <c r="B11" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="15.75">
       <c r="A12" s="9"/>
       <c r="B12" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="15.75">
       <c r="A13" s="9"/>
       <c r="B13" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="15.75">
       <c r="A14" s="9"/>
       <c r="B14" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F14" s="9"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="15.75">
       <c r="A15" s="9"/>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="15.75">
       <c r="A16" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="15.75">
       <c r="A17" s="15"/>
       <c r="B17" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="15.75">
       <c r="A18" s="15"/>
       <c r="B18" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="15.75">
       <c r="A19" s="15"/>
       <c r="B19" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="15.75">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -3242,160 +3250,160 @@
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="15.75">
       <c r="A21" s="9"/>
       <c r="B21" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="15.75">
       <c r="A22" s="9"/>
       <c r="B22" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="15.75">
       <c r="A23" s="9"/>
       <c r="B23" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F23" s="9"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="15.75">
       <c r="A24" s="9"/>
       <c r="B24" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="15.75">
       <c r="A25" s="9"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="15.75">
       <c r="A26" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ht="15.75">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="15.75">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="15.75">
       <c r="A29" s="9"/>
       <c r="B29" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="15.75">
       <c r="A30" s="9"/>
       <c r="B30" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="16"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="15.75">
       <c r="A31" s="9"/>
       <c r="B31" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F31" s="9"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ht="15.75">
       <c r="A32" s="9"/>
       <c r="B32" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C32" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F32" s="9"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="15.75">
       <c r="A33" s="9"/>
       <c r="B33" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="15.75">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3403,56 +3411,56 @@
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="15.75">
       <c r="A35" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
       <c r="E35" s="20"/>
       <c r="F35" s="13"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="15.75">
       <c r="A36" s="21"/>
       <c r="B36" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" ht="15.75">
       <c r="A37" s="21"/>
       <c r="B37" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C37" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E37" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="15.75">
       <c r="A38" s="21"/>
       <c r="B38" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="15.75">
       <c r="A39" s="21"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -3460,44 +3468,44 @@
       <c r="E39" s="22"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ht="15.75">
       <c r="A40" s="21"/>
       <c r="B40" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" ht="15.75">
       <c r="A41" s="21"/>
       <c r="B41" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D41" s="9"/>
       <c r="E41" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F41" s="9"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="15.75">
       <c r="A42" s="21"/>
       <c r="B42" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" ht="15.75">
       <c r="A43" s="21"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -3505,35 +3513,39 @@
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" ht="15.75">
       <c r="A44" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="15.75">
       <c r="A45" s="9"/>
       <c r="F45" s="9"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B47" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
       <c r="B48" t="s">
-        <v>192</v>
-      </c>
-    </row>
+        <v>193</v>
+      </c>
+    </row>
+    <row r="58" ht="15.75"/>
+    <row r="59" ht="15.75"/>
+    <row r="62" ht="15.75"/>
+    <row r="63" ht="15.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3542,217 +3554,217 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29CC185F-F58B-4882-BB6A-99C5A8DAD27D}">
   <dimension ref="A1:J71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.75" customWidth="1"/>
     <col min="2" max="2" width="63" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+    <col min="3" max="3" width="23.375" customWidth="1"/>
+    <col min="4" max="4" width="9.625" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="7" max="7" width="55.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="24" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10"/>
+    <row r="3" spans="1:10">
       <c r="A3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
     </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
     </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="45.75">
       <c r="A8" s="9"/>
       <c r="B8" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
     </row>
-    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10">
       <c r="A10" s="9"/>
       <c r="B10" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="B12" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="15"/>
       <c r="B13" s="25"/>
       <c r="C13" s="25"/>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="A14" s="14" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="G14" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
     </row>
-    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="G15" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
     </row>
-    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="A16" s="9"/>
       <c r="B16" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" s="9"/>
       <c r="B17" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="G17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
       <c r="J17" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3763,347 +3775,347 @@
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10">
       <c r="A19" s="9"/>
       <c r="B19" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="G19" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
     </row>
-    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G20" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
       <c r="B21" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H21" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
       <c r="B22" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G22" s="25"/>
       <c r="H22" s="25"/>
       <c r="J22" s="9"/>
     </row>
-    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10">
       <c r="A23" s="9"/>
       <c r="B23" s="18"/>
       <c r="C23" s="19"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
     </row>
-    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10">
       <c r="A24" s="10" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
       <c r="A25" s="9"/>
     </row>
-    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10">
       <c r="A26" s="9"/>
     </row>
-    <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10">
       <c r="A27" s="9"/>
     </row>
-    <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10">
       <c r="A28" s="9"/>
     </row>
-    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10">
       <c r="A29" s="9"/>
     </row>
-    <row r="30" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10">
       <c r="A30" s="9"/>
     </row>
-    <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10"/>
+    <row r="32" spans="1:10"/>
+    <row r="33" spans="1:5">
       <c r="A33" s="21"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5">
       <c r="A34" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
       <c r="E34" s="20"/>
     </row>
-    <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5">
       <c r="A35" s="21"/>
       <c r="B35" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
     </row>
-    <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5">
       <c r="A36" s="21"/>
       <c r="B36" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
       <c r="A37" s="21"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="22"/>
     </row>
-    <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5">
       <c r="A38" s="21"/>
       <c r="B38" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
     </row>
-    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5">
       <c r="A39" s="21"/>
       <c r="B39" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
       <c r="B40" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5">
       <c r="A42" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
     </row>
-    <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5">
       <c r="A43" s="9"/>
       <c r="B43" s="16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C43" s="16"/>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
     </row>
-    <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C44" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E44" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
-    <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5">
       <c r="B47" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
     </row>
-    <row r="48" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5">
       <c r="B48" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
       <c r="B49" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C49" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="51" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="52" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5"/>
+    <row r="51" spans="1:5"/>
+    <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B52" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
       <c r="D53" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B54" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5"/>
+    <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B56" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
       <c r="B57" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B58" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D58" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E58" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5"/>
+    <row r="60" spans="1:5">
       <c r="D60" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="62" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="63" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="64" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="65" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="16" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="16" x14ac:dyDescent="0.2"/>
+        <v>228</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5"/>
+    <row r="62" spans="1:5"/>
+    <row r="63" spans="1:5"/>
+    <row r="64" spans="1:5"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4112,43 +4124,43 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C5580AA-63C5-4A17-B275-34DB10D89DEB}">
   <dimension ref="A14:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="52.33203125" customWidth="1"/>
+    <col min="1" max="1" width="52.375" customWidth="1"/>
     <col min="2" max="2" width="35.5" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75">
       <c r="A16" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C16" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C18" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>235</v>
+      </c>
+      <c r="C19" t="s">
         <v>234</v>
-      </c>
-      <c r="C19" t="s">
-        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -4162,27 +4174,27 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08672E17-9FFE-4DB4-AF66-56E8BA384E79}">
   <dimension ref="A14:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="24.1640625" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.1640625" customWidth="1"/>
+    <col min="1" max="1" width="24.25" customWidth="1"/>
+    <col min="2" max="2" width="14.875" customWidth="1"/>
+    <col min="4" max="4" width="22.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -4193,7 +4205,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11C2D4C5-F861-4F4B-9751-7CF6281C8800}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.95"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4209,12 +4221,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100411B9ADA3C88D84DA852962C88CCCF71" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fb8c17446f1b3f0664823c0cd0cfd6e0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="29555bce-99f7-4351-a06e-6e58a2a8a9c5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a69d9eff398ae5b3f2ca614c38d74f66" ns2:_="">
     <xsd:import namespace="29555bce-99f7-4351-a06e-6e58a2a8a9c5"/>
@@ -4352,37 +4358,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C57BA70C-BAC7-4091-B4F1-876342C6970D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C57BA70C-BAC7-4091-B4F1-876342C6970D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="29555bce-99f7-4351-a06e-6e58a2a8a9c5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}"/>
 </file>
</xml_diff>

<commit_message>
fix duplicate --by block
</commit_message>
<xml_diff>
--- a/curriculum-2026.xlsx
+++ b/curriculum-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chunbeiwang\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pragatidahal/dspg-2026-curriculum-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1173" documentId="13_ncr:1_{65F6ACF4-0E11-4456-A716-D1BBD8106E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31698AAF-FD04-4466-9B80-BC349D3B273E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB06B30C-810C-2044-AB7A-3DF4D8D3A484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15980" yWindow="580" windowWidth="20680" windowHeight="20730" firstSheet="5" activeTab="5" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
+    <workbookView xWindow="8120" yWindow="600" windowWidth="20680" windowHeight="16100" xr2:uid="{53A63D6F-E822-9F49-8454-1C6D116A7C22}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -60,9 +60,6 @@
     <t>Week 1</t>
   </si>
   <si>
-    <t>Onboarding and Basic Research skills</t>
-  </si>
-  <si>
     <t>Onboarding and Project Assignment</t>
   </si>
   <si>
@@ -776,12 +773,15 @@
   <si>
     <t>Timing : 9 - 11</t>
   </si>
+  <si>
+    <t>Onboarding and Basic Research skills</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -814,28 +814,31 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
@@ -849,6 +852,7 @@
       <sz val="12"/>
       <color rgb="FF242424"/>
       <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1301,17 +1305,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85F7D784-1E42-A348-A9E2-F410F7914403}">
   <dimension ref="A2:D22"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.625" style="1"/>
-    <col min="2" max="2" width="61.75" style="1" customWidth="1"/>
-    <col min="3" max="3" width="48.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.25" style="1" customWidth="1"/>
-    <col min="5" max="5" width="47.875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.625" style="1"/>
+    <col min="1" max="1" width="10.6640625" style="1"/>
+    <col min="2" max="2" width="61.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="48.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47.83203125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1322,108 +1326,108 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="1" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="1" t="s">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="1" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="1" t="s">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="1" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="1" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="1" t="s">
+    </row>
+    <row r="22" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="30.75">
-      <c r="A22" s="1" t="s">
+      <c r="B22" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1437,7 +1441,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D97929D-AD65-4CE9-BF8E-66086023685B}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1446,7 +1450,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74299BF2-7816-4D37-8F2E-A4AEC8FE33CF}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1455,51 +1459,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79ABCE58-A8F1-4047-AD55-074F18A4BD46}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.25" style="9" customWidth="1"/>
-    <col min="2" max="2" width="72.125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="18.75" style="9" customWidth="1"/>
-    <col min="4" max="4" width="16.125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="40.75" style="9" customWidth="1"/>
-    <col min="6" max="6" width="13.75" style="9" customWidth="1"/>
-    <col min="7" max="16384" width="10.625" style="9"/>
+    <col min="1" max="1" width="21.1640625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="72.1640625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="40.6640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" style="9" customWidth="1"/>
+    <col min="7" max="16384" width="10.6640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="8"/>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="9" t="s">
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="C4" s="12">
         <v>0.52083333333333337</v>
@@ -1508,139 +1512,139 @@
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6"/>
-    <row r="6" spans="1:6">
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>40</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="8" spans="1:6" ht="21.75" customHeight="1">
+    <row r="8" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>41</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>42</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
     </row>
-    <row r="9" spans="1:6" ht="21.75" customHeight="1">
+    <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="15"/>
       <c r="B9" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" ht="148.5" customHeight="1">
+    <row r="10" spans="1:6" ht="148.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="15"/>
       <c r="B10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="E10" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="18" t="s">
+    </row>
+    <row r="11" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="18" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="33" customHeight="1">
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="E11" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="9" t="s">
+    </row>
+    <row r="12" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="9" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="19.5" customHeight="1">
-      <c r="B12" s="9" t="s">
+      <c r="C12" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="9" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="16" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" customHeight="1"/>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1">
-      <c r="B14" s="16" t="s">
-        <v>53</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="E15" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E15" s="9" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="18" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="63" customHeight="1">
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="20.25" customHeight="1">
+    </row>
+    <row r="17" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18"/>
       <c r="C17" s="19"/>
     </row>
-    <row r="18" spans="1:7" ht="21" customHeight="1">
+    <row r="18" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>60</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>61</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="13" t="s">
         <v>62</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="20"/>
       <c r="F20" s="13"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="21"/>
       <c r="B21" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -1648,183 +1652,183 @@
       <c r="F21" s="16"/>
       <c r="G21" s="21"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="21"/>
       <c r="B22" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" s="21"/>
       <c r="E22" s="21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="21"/>
       <c r="B23" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="E23" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E23" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="21"/>
       <c r="B24" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="E24" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="E24" s="27" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+    </row>
+    <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="21"/>
       <c r="E25" s="22"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="21"/>
       <c r="B26" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
       <c r="F26" s="16"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="21"/>
       <c r="B27" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="21"/>
       <c r="B28" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="21"/>
+    </row>
+    <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="21"/>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="10" t="s">
+      <c r="B30" s="13" t="s">
         <v>74</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>75</v>
       </c>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B31" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="B32" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="E32" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E32" s="9" t="s">
+    </row>
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B33" s="9" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="B33" s="9" t="s">
-        <v>79</v>
-      </c>
       <c r="E33" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6"/>
-    <row r="35" spans="1:6" ht="15.75" customHeight="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="B36" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="E36" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E36" s="9" t="s">
+    </row>
+    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B37" s="9" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="B37" s="9" t="s">
+      <c r="C37" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="E37" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B38" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E37" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="B38" s="9" t="s">
+      <c r="C38" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="E38" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="B39" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="E38" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="B39" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C39" s="9" t="s">
+    </row>
+    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="9" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="40" spans="1:6"/>
-    <row r="41" spans="1:6">
-      <c r="A41" s="9" t="s">
+      <c r="B41" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B41" s="9" t="s">
+    </row>
+    <row r="42" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B42" s="9" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.75" customHeight="1">
-      <c r="B42" s="9" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1835,96 +1839,95 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E724203-93BF-4AB3-BBFF-F621604F3060}">
   <dimension ref="A1:M57"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.625" customWidth="1"/>
-    <col min="2" max="2" width="65.375" customWidth="1"/>
-    <col min="3" max="3" width="18.75" customWidth="1"/>
-    <col min="5" max="5" width="41.625" customWidth="1"/>
-    <col min="6" max="6" width="10.625" customWidth="1"/>
-    <col min="9" max="9" width="30.625" customWidth="1"/>
-    <col min="12" max="12" width="20.75" customWidth="1"/>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="65.33203125" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="41.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" customWidth="1"/>
+    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="12" max="12" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75"/>
-    <row r="3" spans="1:6" ht="15.75">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17.25" customHeight="1">
+    <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>93</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>94</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75">
+    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -1932,45 +1935,45 @@
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -1978,59 +1981,59 @@
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75">
+    <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="15"/>
       <c r="B14" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:13" ht="15.75">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -2038,45 +2041,45 @@
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:13" ht="15.75">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
     </row>
-    <row r="19" spans="1:13" ht="15.75">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:13" ht="15.75">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:13" ht="15.75">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="18"/>
       <c r="C21" s="19"/>
@@ -2084,12 +2087,12 @@
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:13" ht="15.75">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>108</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>109</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -2097,47 +2100,47 @@
       <c r="F22" s="13"/>
       <c r="M22" s="3"/>
     </row>
-    <row r="23" spans="1:13" ht="15.75">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
     </row>
-    <row r="24" spans="1:13" ht="15.75">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:13" ht="15.75">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:13" ht="15.75">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -2145,45 +2148,45 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:13" ht="15.75">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:13" ht="15.75">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:13" ht="15.75">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:13" ht="15.75">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -2191,12 +2194,12 @@
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:13" ht="15.75">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>112</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>113</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
@@ -2204,48 +2207,48 @@
       <c r="F31" s="13"/>
       <c r="M31" s="3"/>
     </row>
-    <row r="32" spans="1:13" ht="15.75">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="21"/>
       <c r="B32" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:13" ht="15.75">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D33" s="21"/>
       <c r="E33" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F33" s="21"/>
       <c r="M33" s="3"/>
     </row>
-    <row r="34" spans="1:13" ht="15.75">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="21"/>
       <c r="B34" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="E34" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="E34" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:13" ht="18.75" customHeight="1">
+    <row r="35" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -2254,45 +2257,45 @@
       <c r="F35" s="9"/>
       <c r="M35" s="3"/>
     </row>
-    <row r="36" spans="1:13" ht="15.75">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:13" ht="15.75">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:13" ht="15.75">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:13" ht="15.75">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -2300,85 +2303,85 @@
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40" spans="1:13" ht="15.75">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B40" s="13" t="s">
         <v>117</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>118</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
     </row>
-    <row r="41" spans="1:13" ht="15.75">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
       <c r="F41" s="16"/>
     </row>
-    <row r="42" spans="1:13" ht="15.75">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="9"/>
       <c r="B42" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D42" s="21"/>
       <c r="E42" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:13" ht="15.75">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>120</v>
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:13" ht="15.75">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C44" s="9" t="s">
         <v>122</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>123</v>
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F44" s="9"/>
     </row>
-    <row r="45" spans="1:13" ht="15.75">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C45" s="9" t="s">
         <v>125</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>126</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F45" s="9"/>
     </row>
-    <row r="46" spans="1:13" ht="15.75">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
@@ -2386,86 +2389,84 @@
       <c r="E46" s="9"/>
       <c r="F46" s="9"/>
     </row>
-    <row r="47" spans="1:13" ht="15.75">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="9"/>
       <c r="B47" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
       <c r="F47" s="16"/>
     </row>
-    <row r="48" spans="1:13" ht="15.75">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="9"/>
       <c r="B48" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F48" s="9"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B49" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C49" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E48" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F48" s="9"/>
-    </row>
-    <row r="49" spans="1:5" ht="15.75">
-      <c r="B49" s="9" t="s">
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B50" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="15.75">
-      <c r="B50" s="9" t="s">
-        <v>129</v>
-      </c>
       <c r="C50" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="15.75">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B51" s="9" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="15.75">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B52" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>130</v>
       </c>
-      <c r="C52" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="15.75"/>
-    <row r="54" spans="1:5" ht="15.75"/>
-    <row r="55" spans="1:5" ht="15.75">
-      <c r="A55" t="s">
+      <c r="B55" t="s">
         <v>131</v>
       </c>
-      <c r="B55" t="s">
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.75">
-      <c r="B56" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5">
-      <c r="B57" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2475,107 +2476,107 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4375F624-6CA8-4BD1-8837-D674A15E3640}">
-  <dimension ref="A1:F85"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <dimension ref="A1:F67"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.25" customWidth="1"/>
-    <col min="2" max="2" width="68.375" customWidth="1"/>
-    <col min="3" max="3" width="21.75" customWidth="1"/>
+    <col min="1" max="1" width="33.1640625" customWidth="1"/>
+    <col min="2" max="2" width="68.33203125" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="42.875" customWidth="1"/>
-    <col min="6" max="6" width="14.625" customWidth="1"/>
+    <col min="5" max="5" width="42.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15.75">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75">
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>136</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>137</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75">
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="26" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -2583,97 +2584,97 @@
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F11" s="9"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="B13" s="25"/>
       <c r="C13" s="25"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75">
+    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>148</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>149</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="C16" s="29" t="s">
         <v>150</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>151</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:6" ht="15.75">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
     </row>
-    <row r="18" spans="1:6" ht="15.75">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -2681,44 +2682,44 @@
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" ht="15.75">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" ht="15.75">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F21" s="9"/>
     </row>
-    <row r="22" spans="1:6" ht="15.75">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="9"/>
       <c r="B22" s="18"/>
       <c r="C22" s="19"/>
@@ -2726,43 +2727,43 @@
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>153</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
     </row>
-    <row r="24" spans="1:6" ht="15.75">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
     </row>
-    <row r="25" spans="1:6" ht="15.75">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:6" ht="15.75">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -2770,44 +2771,44 @@
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:6" ht="15.75">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:6" ht="15.75">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" ht="15.75">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" ht="15.75">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -2815,43 +2816,43 @@
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:6" ht="15.75">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>156</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>157</v>
       </c>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
       <c r="E31" s="20"/>
       <c r="F31" s="13"/>
     </row>
-    <row r="32" spans="1:6" ht="15.75">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="21"/>
       <c r="B32" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:6" ht="15.75">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="21"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -2859,44 +2860,44 @@
       <c r="E34" s="22"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F36" s="9"/>
     </row>
-    <row r="37" spans="1:6" ht="15.75">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -2904,56 +2905,56 @@
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B39" s="13" t="s">
         <v>160</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>161</v>
       </c>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
     </row>
-    <row r="40" spans="1:6" ht="15.75">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="9"/>
       <c r="B40" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
     </row>
-    <row r="41" spans="1:6" ht="15.75">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
+        <v>161</v>
+      </c>
+      <c r="C41" t="s">
         <v>162</v>
       </c>
-      <c r="C41" t="s">
-        <v>163</v>
-      </c>
       <c r="E41" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F41" s="9"/>
     </row>
-    <row r="42" spans="1:6" ht="15.75">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="9"/>
       <c r="B42" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:6" ht="15.75">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -2961,57 +2962,52 @@
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" ht="15.75">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C44" s="16"/>
       <c r="D44" s="16"/>
       <c r="E44" s="16"/>
       <c r="F44" s="16"/>
     </row>
-    <row r="45" spans="1:6" ht="15.75">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C45" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F45" s="9"/>
     </row>
-    <row r="46" spans="1:6" ht="15.75">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B46" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="15.75">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="B49" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="B49" s="25" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2" ht="15.75">
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" s="4"/>
     </row>
-    <row r="78" spans="2:2" ht="15.75"/>
-    <row r="79" spans="2:2" ht="15.75"/>
-    <row r="80" spans="2:2" ht="15.75"/>
-    <row r="84" ht="15.75"/>
-    <row r="85" ht="15.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3019,119 +3015,119 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E959A69-B699-4CFA-82E0-7BD72875D037}">
-  <dimension ref="A1:F63"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.375" customWidth="1"/>
+    <col min="1" max="1" width="27.33203125" customWidth="1"/>
     <col min="2" max="2" width="58.5" customWidth="1"/>
-    <col min="3" max="3" width="17.625" customWidth="1"/>
-    <col min="4" max="4" width="9.375" customWidth="1"/>
-    <col min="5" max="5" width="32.625" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="24"/>
     </row>
-    <row r="3" spans="1:6" ht="15.75">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="25" t="s">
         <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75">
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>169</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>170</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" ht="15.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" ht="15.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F6" s="9"/>
     </row>
-    <row r="7" spans="1:6" ht="15.75">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F7" s="9"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75">
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>171</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>172</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F8" s="9"/>
     </row>
-    <row r="9" spans="1:6" ht="15.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
-    <row r="10" spans="1:6" ht="15.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -3139,110 +3135,110 @@
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
     </row>
-    <row r="12" spans="1:6" ht="15.75">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F12" s="9"/>
     </row>
-    <row r="13" spans="1:6" ht="15.75">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="B13" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F13" s="9"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
       <c r="B14" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" s="9"/>
     </row>
-    <row r="15" spans="1:6" ht="15.75">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
     </row>
-    <row r="16" spans="1:6" ht="15.75">
+    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="B16" s="23" t="s">
         <v>176</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>177</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
     </row>
-    <row r="17" spans="1:6" ht="15.75">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
     </row>
-    <row r="18" spans="1:6" ht="15.75">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="15"/>
       <c r="B18" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" ht="15.75">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="15"/>
       <c r="B19" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -3250,160 +3246,160 @@
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" ht="15.75">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
     </row>
-    <row r="22" spans="1:6" ht="15.75">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="9"/>
       <c r="B22" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F23" s="9"/>
     </row>
-    <row r="24" spans="1:6" ht="15.75">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
       <c r="B24" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:6" ht="15.75">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
     </row>
-    <row r="26" spans="1:6" ht="15.75">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>181</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>182</v>
       </c>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
     </row>
-    <row r="27" spans="1:6" ht="15.75">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
       <c r="B27" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
     </row>
-    <row r="28" spans="1:6" ht="15.75">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
       <c r="B28" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" ht="15.75">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
       <c r="B29" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
     </row>
-    <row r="30" spans="1:6" ht="15.75">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
       <c r="B30" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="16"/>
     </row>
-    <row r="31" spans="1:6" ht="15.75">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="9"/>
       <c r="B31" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F31" s="9"/>
     </row>
-    <row r="32" spans="1:6" ht="15.75">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="9"/>
       <c r="B32" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F32" s="9"/>
     </row>
-    <row r="33" spans="1:6" ht="15.75">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="9"/>
       <c r="B33" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3411,56 +3407,56 @@
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
     </row>
-    <row r="35" spans="1:6" ht="15.75">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B35" s="13" t="s">
         <v>186</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>187</v>
       </c>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
       <c r="E35" s="20"/>
       <c r="F35" s="13"/>
     </row>
-    <row r="36" spans="1:6" ht="15.75">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:6" ht="15.75">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s">
         <v>162</v>
       </c>
-      <c r="C37" t="s">
-        <v>163</v>
-      </c>
       <c r="E37" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F37" s="9"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F38" s="9"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -3468,44 +3464,44 @@
       <c r="E39" s="22"/>
       <c r="F39" s="9"/>
     </row>
-    <row r="40" spans="1:6" ht="15.75">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="21"/>
       <c r="B40" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
     </row>
-    <row r="41" spans="1:6" ht="15.75">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="21"/>
       <c r="B41" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D41" s="9"/>
       <c r="E41" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F41" s="9"/>
     </row>
-    <row r="42" spans="1:6" ht="15.75">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="21"/>
       <c r="B42" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F42" s="9"/>
     </row>
-    <row r="43" spans="1:6" ht="15.75">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="21"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -3513,39 +3509,35 @@
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
     </row>
-    <row r="44" spans="1:6" ht="15.75">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="B44" s="13" t="s">
         <v>189</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>190</v>
       </c>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
     </row>
-    <row r="45" spans="1:6" ht="15.75">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="F45" s="9"/>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>190</v>
+      </c>
+      <c r="B47" t="s">
         <v>191</v>
       </c>
-      <c r="B47" t="s">
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
-      <c r="B48" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="58" ht="15.75"/>
-    <row r="59" ht="15.75"/>
-    <row r="62" ht="15.75"/>
-    <row r="63" ht="15.75"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3554,217 +3546,217 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29CC185F-F58B-4882-BB6A-99C5A8DAD27D}">
   <dimension ref="A1:J71"/>
-  <sheetFormatPr defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.75" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
     <col min="2" max="2" width="63" customWidth="1"/>
-    <col min="3" max="3" width="23.375" customWidth="1"/>
-    <col min="4" max="4" width="9.625" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="7" max="7" width="55.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="2" spans="1:10"/>
-    <row r="3" spans="1:10">
-      <c r="A3" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="10" t="s">
+      <c r="B4" s="23" t="s">
         <v>195</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>196</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="9"/>
       <c r="B5" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>139</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
       <c r="B7" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>197</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>198</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="45.75">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="9"/>
       <c r="B10" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B12" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
       <c r="B13" s="25"/>
       <c r="C13" s="25"/>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>202</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>203</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="G14" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="G15" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="9"/>
       <c r="B16" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>205</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>206</v>
       </c>
       <c r="D16" s="9"/>
       <c r="E16" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="G16" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>208</v>
-      </c>
       <c r="H16" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="B17" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="G17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
       <c r="J17" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -3775,347 +3767,347 @@
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="G19" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H21" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B22" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G22" s="25"/>
       <c r="H22" s="25"/>
       <c r="J22" s="9"/>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="9"/>
       <c r="B23" s="18"/>
       <c r="C23" s="19"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="9"/>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="9"/>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="9"/>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="9"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="9"/>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="9"/>
     </row>
-    <row r="31" spans="1:10"/>
-    <row r="32" spans="1:10"/>
-    <row r="33" spans="1:5">
+    <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>213</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>214</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
       <c r="E34" s="20"/>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="22"/>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C39" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B40" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="9"/>
       <c r="B43" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C43" s="16"/>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
+        <v>161</v>
+      </c>
+      <c r="C44" t="s">
         <v>162</v>
       </c>
-      <c r="C44" t="s">
-        <v>163</v>
-      </c>
       <c r="E44" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B47" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B48" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C48" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="25" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C49" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5"/>
-    <row r="51" spans="1:5"/>
-    <row r="52" spans="1:5">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="51" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="52" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>215</v>
+      </c>
+      <c r="B52" t="s">
         <v>216</v>
       </c>
-      <c r="B52" t="s">
+    </row>
+    <row r="53" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="D53" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
-      <c r="D53" t="s">
+    <row r="54" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" t="s">
+      <c r="B54" t="s">
         <v>219</v>
       </c>
-      <c r="B54" t="s">
+    </row>
+    <row r="55" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="55" spans="1:5"/>
-    <row r="56" spans="1:5">
-      <c r="A56" t="s">
+      <c r="B56" t="s">
         <v>221</v>
       </c>
-      <c r="B56" t="s">
+    </row>
+    <row r="57" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
-      <c r="B57" t="s">
+    <row r="58" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
-      <c r="A58" t="s">
+      <c r="B58" t="s">
         <v>224</v>
       </c>
-      <c r="B58" t="s">
+      <c r="D58" t="s">
         <v>225</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>226</v>
       </c>
-      <c r="E58" t="s">
+    </row>
+    <row r="59" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="D60" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="59" spans="1:5"/>
-    <row r="60" spans="1:5">
-      <c r="D60" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5"/>
-    <row r="62" spans="1:5"/>
-    <row r="63" spans="1:5"/>
-    <row r="64" spans="1:5"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
+    <row r="61" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="62" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="63" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="1:5" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="65" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="66" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="67" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="69" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="70" ht="16" x14ac:dyDescent="0.2"/>
+    <row r="71" ht="16" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4124,43 +4116,43 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C5580AA-63C5-4A17-B275-34DB10D89DEB}">
   <dimension ref="A14:C19"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="52.375" customWidth="1"/>
+    <col min="1" max="1" width="52.33203125" customWidth="1"/>
     <col min="2" max="2" width="35.5" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.75">
-      <c r="A16" t="s">
+      <c r="B16" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="C16" t="s">
         <v>231</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
+      <c r="C18" t="s">
         <v>233</v>
       </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>235</v>
-      </c>
       <c r="C19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -4174,27 +4166,27 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08672E17-9FFE-4DB4-AF66-56E8BA384E79}">
   <dimension ref="A14:D15"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.25" customWidth="1"/>
-    <col min="2" max="2" width="14.875" customWidth="1"/>
-    <col min="4" max="4" width="22.125" customWidth="1"/>
+    <col min="1" max="1" width="24.1640625" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>235</v>
+      </c>
+      <c r="B15" t="s">
+        <v>216</v>
+      </c>
+      <c r="D15" t="s">
         <v>236</v>
-      </c>
-      <c r="B15" t="s">
-        <v>217</v>
-      </c>
-      <c r="D15" t="s">
-        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -4205,7 +4197,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11C2D4C5-F861-4F4B-9751-7CF6281C8800}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4365,13 +4357,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E948F4DD-3F9E-4963-820A-2F7ED559FDDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C57BA70C-BAC7-4091-B4F1-876342C6970D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C57BA70C-BAC7-4091-B4F1-876342C6970D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="29555bce-99f7-4351-a06e-6e58a2a8a9c5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6B2C08C-1A19-45F4-B774-B4C06928DC26}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>